<commit_message>
qwen3.5:9b plain COT results generated
</commit_message>
<xml_diff>
--- a/results/qwen3_5_9b/comparison_CoTPlainLLM/CoTPlainLLM_costs.xlsx
+++ b/results/qwen3_5_9b/comparison_CoTPlainLLM/CoTPlainLLM_costs.xlsx
@@ -472,16 +472,16 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.001750946044921875</v>
+        <v>115.191154718399</v>
       </c>
       <c r="B2" t="n">
-        <v>1137.546875</v>
+        <v>1122.41015625</v>
       </c>
       <c r="C2" t="n">
-        <v>8.9</v>
+        <v>11.7</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -490,7 +490,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0.001747608184814453</v>
+        <v>115.191150188446</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -498,16 +498,16 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.0007207393646240234</v>
+        <v>13.92340135574341</v>
       </c>
       <c r="B3" t="n">
-        <v>1137.546875</v>
+        <v>1122.4140625</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>13.9</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -516,7 +516,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0007185935974121094</v>
+        <v>13.92339706420898</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -524,16 +524,16 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.0005638599395751953</v>
+        <v>12.34152984619141</v>
       </c>
       <c r="B4" t="n">
-        <v>1137.546875</v>
+        <v>1122.421875</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -542,7 +542,7 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0005629062652587891</v>
+        <v>12.34152793884277</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -550,16 +550,16 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.0005657672882080078</v>
+        <v>88.45020294189453</v>
       </c>
       <c r="B5" t="n">
-        <v>1137.546875</v>
+        <v>1122.484375</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -568,7 +568,7 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0005645751953125</v>
+        <v>88.45020151138306</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -576,16 +576,16 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.0005598068237304688</v>
+        <v>13.12002301216125</v>
       </c>
       <c r="B6" t="n">
-        <v>1137.546875</v>
+        <v>1122.48828125</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -594,7 +594,7 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0005581378936767578</v>
+        <v>13.1200213432312</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -602,16 +602,16 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.0006213188171386719</v>
+        <v>46.72975134849548</v>
       </c>
       <c r="B7" t="n">
-        <v>1137.5703125</v>
+        <v>1122.52734375</v>
       </c>
       <c r="C7" t="n">
-        <v>50</v>
+        <v>13.6</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -620,7 +620,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0006203651428222656</v>
+        <v>46.72974967956543</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -628,16 +628,16 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.0006301403045654297</v>
+        <v>27.93844819068909</v>
       </c>
       <c r="B8" t="n">
-        <v>1137.58984375</v>
+        <v>1122.55859375</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>14.2</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -646,7 +646,7 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0006289482116699219</v>
+        <v>27.93844604492188</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -654,16 +654,16 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.0005536079406738281</v>
+        <v>20.03808856010437</v>
       </c>
       <c r="B9" t="n">
-        <v>1137.59765625</v>
+        <v>1122.55859375</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -672,7 +672,7 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0005524158477783203</v>
+        <v>20.03808641433716</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -680,16 +680,16 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.0005965232849121094</v>
+        <v>19.79366898536682</v>
       </c>
       <c r="B10" t="n">
-        <v>1137.61328125</v>
+        <v>1122.578125</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>14.3</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -698,7 +698,7 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0005953311920166016</v>
+        <v>19.79366707801819</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
@@ -706,16 +706,16 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.0007634162902832031</v>
+        <v>22.68939542770386</v>
       </c>
       <c r="B11" t="n">
-        <v>1137.61328125</v>
+        <v>1122.59375</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>13.5</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -724,7 +724,7 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0007624626159667969</v>
+        <v>22.68939328193665</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -732,16 +732,16 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.000568389892578125</v>
+        <v>29.53063464164734</v>
       </c>
       <c r="B12" t="n">
-        <v>1137.61328125</v>
+        <v>1122.625</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>14.6</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
@@ -750,7 +750,7 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0005671977996826172</v>
+        <v>29.53063297271729</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -758,16 +758,16 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.0005335807800292969</v>
+        <v>4931.92600607872</v>
       </c>
       <c r="B13" t="n">
-        <v>1137.61328125</v>
+        <v>1127.90625</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>14.1</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -776,7 +776,7 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0005326271057128906</v>
+        <v>4931.926004171371</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -784,16 +784,16 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.0005657672882080078</v>
+        <v>24.44480681419373</v>
       </c>
       <c r="B14" t="n">
-        <v>1137.6171875</v>
+        <v>1127.90625</v>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>13.6</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
@@ -802,7 +802,7 @@
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0005645751953125</v>
+        <v>24.44480490684509</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -810,16 +810,16 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.0005266666412353516</v>
+        <v>14.39043784141541</v>
       </c>
       <c r="B15" t="n">
-        <v>1137.6171875</v>
+        <v>1127.90625</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>14.7</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -828,7 +828,7 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0005254745483398438</v>
+        <v>14.39043545722961</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -836,16 +836,16 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.0005431175231933594</v>
+        <v>38.47407674789429</v>
       </c>
       <c r="B16" t="n">
-        <v>1137.62109375</v>
+        <v>1127.90625</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>14.1</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -854,7 +854,7 @@
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0005421638488769531</v>
+        <v>38.47407412528992</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -862,16 +862,16 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.0006074905395507812</v>
+        <v>19.70282649993896</v>
       </c>
       <c r="B17" t="n">
-        <v>1137.63671875</v>
+        <v>1127.90625</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>13.3</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -880,7 +880,7 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>0.0006062984466552734</v>
+        <v>19.70282483100891</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -888,16 +888,16 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.0005686283111572266</v>
+        <v>30.20188903808594</v>
       </c>
       <c r="B18" t="n">
-        <v>1137.63671875</v>
+        <v>1127.90625</v>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>14.2</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
@@ -906,7 +906,7 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0005674362182617188</v>
+        <v>30.20188736915588</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
@@ -914,16 +914,16 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.0007686614990234375</v>
+        <v>16.33299970626831</v>
       </c>
       <c r="B19" t="n">
-        <v>1137.640625</v>
+        <v>1127.90625</v>
       </c>
       <c r="C19" t="n">
-        <v>4.8</v>
+        <v>14.5</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
@@ -932,7 +932,7 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>0.0007674694061279297</v>
+        <v>16.33299708366394</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
@@ -940,16 +940,16 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0.0005745887756347656</v>
+        <v>21.87162399291992</v>
       </c>
       <c r="B20" t="n">
-        <v>1137.640625</v>
+        <v>1127.90625</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>13.4</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -958,7 +958,7 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>0.0005731582641601562</v>
+        <v>21.87162113189697</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -966,16 +966,16 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.0007383823394775391</v>
+        <v>73.41635632514954</v>
       </c>
       <c r="B21" t="n">
-        <v>1137.671875</v>
+        <v>1127.90625</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -984,7 +984,7 @@
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0007371902465820312</v>
+        <v>73.41635465621948</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -992,16 +992,16 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0.0005793571472167969</v>
+        <v>26.12026643753052</v>
       </c>
       <c r="B22" t="n">
-        <v>1137.67578125</v>
+        <v>1127.91015625</v>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>13.8</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
@@ -1010,7 +1010,7 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>0.0005781650543212891</v>
+        <v>26.12026476860046</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -1018,16 +1018,16 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0.0005640983581542969</v>
+        <v>31.25837922096252</v>
       </c>
       <c r="B23" t="n">
-        <v>1137.67578125</v>
+        <v>1127.91015625</v>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>14.3</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1036,7 +1036,7 @@
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0005626678466796875</v>
+        <v>31.25837731361389</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -1044,16 +1044,16 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>0.0005233287811279297</v>
+        <v>14.42015266418457</v>
       </c>
       <c r="B24" t="n">
-        <v>1137.67578125</v>
+        <v>1127.9140625</v>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
+        <v>14.1</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1062,7 +1062,7 @@
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>0.0005223751068115234</v>
+        <v>14.42015051841736</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -1070,16 +1070,16 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0.0005159378051757812</v>
+        <v>16.46011018753052</v>
       </c>
       <c r="B25" t="n">
-        <v>1137.67578125</v>
+        <v>1127.9140625</v>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>13.5</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
@@ -1088,7 +1088,7 @@
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>0.000514984130859375</v>
+        <v>16.46010804176331</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1096,16 +1096,16 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>0.0005185604095458984</v>
+        <v>14.32778668403625</v>
       </c>
       <c r="B26" t="n">
-        <v>1137.67578125</v>
+        <v>1127.9140625</v>
       </c>
       <c r="C26" t="n">
-        <v>0</v>
+        <v>13.8</v>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
@@ -1114,7 +1114,7 @@
         <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>0.0005176067352294922</v>
+        <v>14.32778525352478</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -1122,16 +1122,16 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>0.0005252361297607422</v>
+        <v>13.41952538490295</v>
       </c>
       <c r="B27" t="n">
-        <v>1137.67578125</v>
+        <v>1127.9140625</v>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>13.9</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -1140,7 +1140,7 @@
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>0.0005242824554443359</v>
+        <v>13.41952323913574</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
@@ -1148,16 +1148,16 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>0.0007407665252685547</v>
+        <v>13.53641939163208</v>
       </c>
       <c r="B28" t="n">
-        <v>1137.67578125</v>
+        <v>1127.9140625</v>
       </c>
       <c r="C28" t="n">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -1166,7 +1166,7 @@
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>0.0007393360137939453</v>
+        <v>13.53641724586487</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
@@ -1174,16 +1174,16 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>0.0005474090576171875</v>
+        <v>13.3840434551239</v>
       </c>
       <c r="B29" t="n">
-        <v>1137.67578125</v>
+        <v>1127.9140625</v>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>13.9</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
@@ -1192,7 +1192,7 @@
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>0.0005464553833007812</v>
+        <v>13.38404154777527</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -1200,16 +1200,16 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>0.0005505084991455078</v>
+        <v>17.83527374267578</v>
       </c>
       <c r="B30" t="n">
-        <v>1137.67578125</v>
+        <v>1127.9140625</v>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>14.7</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
@@ -1218,7 +1218,7 @@
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0005495548248291016</v>
+        <v>17.83527159690857</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
@@ -1226,16 +1226,16 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>0.0005521774291992188</v>
+        <v>14.47823929786682</v>
       </c>
       <c r="B31" t="n">
-        <v>1137.67578125</v>
+        <v>1127.9140625</v>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>13.9</v>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
@@ -1244,7 +1244,7 @@
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>0.0005507469177246094</v>
+        <v>14.47823691368103</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
@@ -1252,16 +1252,16 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>0.0005581378936767578</v>
+        <v>15.98470735549927</v>
       </c>
       <c r="B32" t="n">
-        <v>1137.67578125</v>
+        <v>1127.9140625</v>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>13.6</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
@@ -1270,7 +1270,7 @@
         <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>0.00055694580078125</v>
+        <v>15.98470568656921</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -1278,16 +1278,16 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>0.0005826950073242188</v>
+        <v>36.12333464622498</v>
       </c>
       <c r="B33" t="n">
-        <v>1137.67578125</v>
+        <v>1127.9140625</v>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>14.2</v>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
@@ -1296,7 +1296,7 @@
         <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>0.0005812644958496094</v>
+        <v>36.12333250045776</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
@@ -1304,16 +1304,16 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>0.0005695819854736328</v>
+        <v>33.4211266040802</v>
       </c>
       <c r="B34" t="n">
-        <v>1137.67578125</v>
+        <v>1127.9140625</v>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>13.6</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
@@ -1322,7 +1322,7 @@
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>0.000568389892578125</v>
+        <v>33.42112469673157</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
@@ -1330,16 +1330,16 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>0.0005662441253662109</v>
+        <v>23.63157033920288</v>
       </c>
       <c r="B35" t="n">
-        <v>1137.67578125</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C35" t="n">
-        <v>0</v>
+        <v>14.2</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
@@ -1348,7 +1348,7 @@
         <v>0</v>
       </c>
       <c r="G35" t="n">
-        <v>0.0005652904510498047</v>
+        <v>23.63156843185425</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
@@ -1356,16 +1356,16 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>0.08188986778259277</v>
+        <v>23.30381035804749</v>
       </c>
       <c r="B36" t="n">
-        <v>1137.67578125</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>14.2</v>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E36" t="n">
         <v>0</v>
@@ -1374,7 +1374,7 @@
         <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>0.08188796043395996</v>
+        <v>23.30380868911743</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
@@ -1382,16 +1382,16 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>0.0007026195526123047</v>
+        <v>58.89286136627197</v>
       </c>
       <c r="B37" t="n">
-        <v>1137.67578125</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C37" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E37" t="n">
         <v>0</v>
@@ -1400,7 +1400,7 @@
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>0.0007009506225585938</v>
+        <v>58.89285969734192</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
@@ -1408,16 +1408,16 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>0.0005817413330078125</v>
+        <v>35.74957013130188</v>
       </c>
       <c r="B38" t="n">
-        <v>1137.67578125</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
+        <v>13.7</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
@@ -1426,7 +1426,7 @@
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>0.0005805492401123047</v>
+        <v>35.74956774711609</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
@@ -1434,16 +1434,16 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>0.0005524158477783203</v>
+        <v>17.68433356285095</v>
       </c>
       <c r="B39" t="n">
-        <v>1137.67578125</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>14.9</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
@@ -1452,7 +1452,7 @@
         <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>0.0005512237548828125</v>
+        <v>17.68433213233948</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -1460,16 +1460,16 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>0.0005397796630859375</v>
+        <v>11.7995457649231</v>
       </c>
       <c r="B40" t="n">
-        <v>1137.67578125</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>13.8</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
         <v>0</v>
       </c>
       <c r="G40" t="n">
-        <v>0.0005383491516113281</v>
+        <v>11.79954361915588</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
@@ -1486,16 +1486,16 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>0.0005390644073486328</v>
+        <v>13.80802798271179</v>
       </c>
       <c r="B41" t="n">
-        <v>1137.67578125</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C41" t="n">
-        <v>50</v>
+        <v>14.3</v>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E41" t="n">
         <v>0</v>
@@ -1504,7 +1504,7 @@
         <v>0</v>
       </c>
       <c r="G41" t="n">
-        <v>0.0005376338958740234</v>
+        <v>13.80802631378174</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
@@ -1512,16 +1512,16 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>0.0005819797515869141</v>
+        <v>12.19240236282349</v>
       </c>
       <c r="B42" t="n">
-        <v>1137.67578125</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C42" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E42" t="n">
         <v>0</v>
@@ -1530,7 +1530,7 @@
         <v>0</v>
       </c>
       <c r="G42" t="n">
-        <v>0.0005807876586914062</v>
+        <v>12.19240069389343</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
@@ -1538,16 +1538,16 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>0.0006234645843505859</v>
+        <v>17.28176188468933</v>
       </c>
       <c r="B43" t="n">
-        <v>1137.6796875</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C43" t="n">
-        <v>0</v>
+        <v>13.6</v>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E43" t="n">
         <v>0</v>
@@ -1556,7 +1556,7 @@
         <v>0</v>
       </c>
       <c r="G43" t="n">
-        <v>0.0006220340728759766</v>
+        <v>17.28175973892212</v>
       </c>
       <c r="H43" t="n">
         <v>0</v>
@@ -1564,16 +1564,16 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>0.0006229877471923828</v>
+        <v>20.63172245025635</v>
       </c>
       <c r="B44" t="n">
-        <v>1137.68359375</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C44" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E44" t="n">
         <v>0</v>
@@ -1582,7 +1582,7 @@
         <v>0</v>
       </c>
       <c r="G44" t="n">
-        <v>0.0006220340728759766</v>
+        <v>20.63172030448914</v>
       </c>
       <c r="H44" t="n">
         <v>0</v>
@@ -1590,16 +1590,16 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>0.0008876323699951172</v>
+        <v>27.26349687576294</v>
       </c>
       <c r="B45" t="n">
-        <v>1137.6875</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C45" t="n">
-        <v>0</v>
+        <v>14.2</v>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E45" t="n">
         <v>0</v>
@@ -1608,7 +1608,7 @@
         <v>0</v>
       </c>
       <c r="G45" t="n">
-        <v>0.0008862018585205078</v>
+        <v>27.26349425315857</v>
       </c>
       <c r="H45" t="n">
         <v>0</v>
@@ -1616,16 +1616,16 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>0.0005619525909423828</v>
+        <v>26.64177870750427</v>
       </c>
       <c r="B46" t="n">
-        <v>1137.69140625</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>13.8</v>
       </c>
       <c r="D46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E46" t="n">
         <v>0</v>
@@ -1634,7 +1634,7 @@
         <v>0</v>
       </c>
       <c r="G46" t="n">
-        <v>0.0005605220794677734</v>
+        <v>26.64177656173706</v>
       </c>
       <c r="H46" t="n">
         <v>0</v>
@@ -1642,16 +1642,16 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>0.0006339550018310547</v>
+        <v>27.7479259967804</v>
       </c>
       <c r="B47" t="n">
-        <v>1137.69921875</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C47" t="n">
-        <v>0</v>
+        <v>13.8</v>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E47" t="n">
         <v>0</v>
@@ -1660,7 +1660,7 @@
         <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>0.0006325244903564453</v>
+        <v>27.74792385101318</v>
       </c>
       <c r="H47" t="n">
         <v>0</v>
@@ -1668,16 +1668,16 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>0.0005788803100585938</v>
+        <v>26.66680431365967</v>
       </c>
       <c r="B48" t="n">
-        <v>1137.69921875</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C48" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E48" t="n">
         <v>0</v>
@@ -1686,7 +1686,7 @@
         <v>0</v>
       </c>
       <c r="G48" t="n">
-        <v>0.0005776882171630859</v>
+        <v>26.66680240631104</v>
       </c>
       <c r="H48" t="n">
         <v>0</v>
@@ -1694,16 +1694,16 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>0.0005807876586914062</v>
+        <v>24.90094685554504</v>
       </c>
       <c r="B49" t="n">
-        <v>1137.69921875</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C49" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E49" t="n">
         <v>0</v>
@@ -1712,7 +1712,7 @@
         <v>0</v>
       </c>
       <c r="G49" t="n">
-        <v>0.0005795955657958984</v>
+        <v>24.90094542503357</v>
       </c>
       <c r="H49" t="n">
         <v>0</v>
@@ -1720,16 +1720,16 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>0.0005800724029541016</v>
+        <v>17.47243642807007</v>
       </c>
       <c r="B50" t="n">
-        <v>1137.703125</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C50" t="n">
-        <v>50</v>
+        <v>13.5</v>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E50" t="n">
         <v>0</v>
@@ -1738,7 +1738,7 @@
         <v>0</v>
       </c>
       <c r="G50" t="n">
-        <v>0.0005791187286376953</v>
+        <v>17.47243428230286</v>
       </c>
       <c r="H50" t="n">
         <v>0</v>
@@ -1746,16 +1746,16 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>0.0005929470062255859</v>
+        <v>18.48544120788574</v>
       </c>
       <c r="B51" t="n">
-        <v>1137.70703125</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C51" t="n">
-        <v>0</v>
+        <v>14.7</v>
       </c>
       <c r="D51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E51" t="n">
         <v>0</v>
@@ -1764,7 +1764,7 @@
         <v>0</v>
       </c>
       <c r="G51" t="n">
-        <v>0.0005919933319091797</v>
+        <v>18.48543906211853</v>
       </c>
       <c r="H51" t="n">
         <v>0</v>
@@ -1772,16 +1772,16 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>0.0006182193756103516</v>
+        <v>17.56378483772278</v>
       </c>
       <c r="B52" t="n">
-        <v>1137.7265625</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C52" t="n">
-        <v>0</v>
+        <v>13.5</v>
       </c>
       <c r="D52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E52" t="n">
         <v>0</v>
@@ -1790,7 +1790,7 @@
         <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>0.0006170272827148438</v>
+        <v>17.56378293037415</v>
       </c>
       <c r="H52" t="n">
         <v>0</v>
@@ -1798,16 +1798,16 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>0.0008375644683837891</v>
+        <v>43.86339092254639</v>
       </c>
       <c r="B53" t="n">
-        <v>1137.74609375</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C53" t="n">
-        <v>0</v>
+        <v>13.8</v>
       </c>
       <c r="D53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E53" t="n">
         <v>0</v>
@@ -1816,7 +1816,7 @@
         <v>0</v>
       </c>
       <c r="G53" t="n">
-        <v>0.0008361339569091797</v>
+        <v>43.86338901519775</v>
       </c>
       <c r="H53" t="n">
         <v>0</v>
@@ -1824,16 +1824,16 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>0.08008384704589844</v>
+        <v>18.37182259559631</v>
       </c>
       <c r="B54" t="n">
-        <v>1137.74609375</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C54" t="n">
-        <v>0</v>
+        <v>14.6</v>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E54" t="n">
         <v>0</v>
@@ -1842,7 +1842,7 @@
         <v>0</v>
       </c>
       <c r="G54" t="n">
-        <v>0.08008217811584473</v>
+        <v>18.37182021141052</v>
       </c>
       <c r="H54" t="n">
         <v>0</v>
@@ -1850,16 +1850,16 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>0.0005624294281005859</v>
+        <v>26.77231502532959</v>
       </c>
       <c r="B55" t="n">
-        <v>1137.74609375</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C55" t="n">
-        <v>50</v>
+        <v>13.9</v>
       </c>
       <c r="D55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E55" t="n">
         <v>0</v>
@@ -1868,7 +1868,7 @@
         <v>0</v>
       </c>
       <c r="G55" t="n">
-        <v>0.0005612373352050781</v>
+        <v>26.77231287956238</v>
       </c>
       <c r="H55" t="n">
         <v>0</v>
@@ -1876,16 +1876,16 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>0.0005567073822021484</v>
+        <v>20.81589031219482</v>
       </c>
       <c r="B56" t="n">
-        <v>1137.74609375</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C56" t="n">
-        <v>0</v>
+        <v>13.9</v>
       </c>
       <c r="D56" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E56" t="n">
         <v>0</v>
@@ -1894,7 +1894,7 @@
         <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>0.0005552768707275391</v>
+        <v>20.81588840484619</v>
       </c>
       <c r="H56" t="n">
         <v>0</v>
@@ -1902,16 +1902,16 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>0.0007112026214599609</v>
+        <v>38.22168803215027</v>
       </c>
       <c r="B57" t="n">
-        <v>1137.76171875</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C57" t="n">
-        <v>0</v>
+        <v>13.9</v>
       </c>
       <c r="D57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E57" t="n">
         <v>0</v>
@@ -1920,7 +1920,7 @@
         <v>0</v>
       </c>
       <c r="G57" t="n">
-        <v>0.0007102489471435547</v>
+        <v>38.22168588638306</v>
       </c>
       <c r="H57" t="n">
         <v>0</v>
@@ -1928,16 +1928,16 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>0.0005829334259033203</v>
+        <v>18.13804960250854</v>
       </c>
       <c r="B58" t="n">
-        <v>1137.76171875</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C58" t="n">
-        <v>0</v>
+        <v>14.2</v>
       </c>
       <c r="D58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E58" t="n">
         <v>0</v>
@@ -1946,7 +1946,7 @@
         <v>0</v>
       </c>
       <c r="G58" t="n">
-        <v>0.0005815029144287109</v>
+        <v>18.13804745674133</v>
       </c>
       <c r="H58" t="n">
         <v>0</v>
@@ -1954,16 +1954,16 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>0.0005910396575927734</v>
+        <v>19.98064231872559</v>
       </c>
       <c r="B59" t="n">
-        <v>1137.765625</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C59" t="n">
-        <v>0</v>
+        <v>13.5</v>
       </c>
       <c r="D59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E59" t="n">
         <v>0</v>
@@ -1972,7 +1972,7 @@
         <v>0</v>
       </c>
       <c r="G59" t="n">
-        <v>0.0005898475646972656</v>
+        <v>19.98063921928406</v>
       </c>
       <c r="H59" t="n">
         <v>0</v>
@@ -1980,16 +1980,16 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>0.0005867481231689453</v>
+        <v>22.38244462013245</v>
       </c>
       <c r="B60" t="n">
-        <v>1137.76953125</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C60" t="n">
-        <v>0</v>
+        <v>14.1</v>
       </c>
       <c r="D60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E60" t="n">
         <v>0</v>
@@ -1998,7 +1998,7 @@
         <v>0</v>
       </c>
       <c r="G60" t="n">
-        <v>0.0005853176116943359</v>
+        <v>22.38244247436523</v>
       </c>
       <c r="H60" t="n">
         <v>0</v>
@@ -2006,16 +2006,16 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>0.0005545616149902344</v>
+        <v>27.77073860168457</v>
       </c>
       <c r="B61" t="n">
-        <v>1137.7734375</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C61" t="n">
-        <v>50</v>
+        <v>13.9</v>
       </c>
       <c r="D61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E61" t="n">
         <v>0</v>
@@ -2024,7 +2024,7 @@
         <v>0</v>
       </c>
       <c r="G61" t="n">
-        <v>0.000553131103515625</v>
+        <v>27.77073621749878</v>
       </c>
       <c r="H61" t="n">
         <v>0</v>
@@ -2032,16 +2032,16 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>0.0007710456848144531</v>
+        <v>13.80406355857849</v>
       </c>
       <c r="B62" t="n">
-        <v>1137.7734375</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C62" t="n">
-        <v>0</v>
+        <v>13.9</v>
       </c>
       <c r="D62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E62" t="n">
         <v>0</v>
@@ -2050,7 +2050,7 @@
         <v>0</v>
       </c>
       <c r="G62" t="n">
-        <v>0.0007700920104980469</v>
+        <v>13.80405926704407</v>
       </c>
       <c r="H62" t="n">
         <v>0</v>
@@ -2058,16 +2058,16 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>0.0005686283111572266</v>
+        <v>14.48620676994324</v>
       </c>
       <c r="B63" t="n">
-        <v>1137.7734375</v>
+        <v>1127.91796875</v>
       </c>
       <c r="C63" t="n">
-        <v>0</v>
+        <v>14.7</v>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E63" t="n">
         <v>0</v>
@@ -2076,7 +2076,7 @@
         <v>0</v>
       </c>
       <c r="G63" t="n">
-        <v>0.0005674362182617188</v>
+        <v>14.48620438575745</v>
       </c>
       <c r="H63" t="n">
         <v>0</v>
@@ -2084,16 +2084,16 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>0.0005724430084228516</v>
+        <v>18.41884517669678</v>
       </c>
       <c r="B64" t="n">
-        <v>1137.7734375</v>
+        <v>1127.921875</v>
       </c>
       <c r="C64" t="n">
-        <v>0</v>
+        <v>14.1</v>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E64" t="n">
         <v>0</v>
@@ -2102,7 +2102,7 @@
         <v>0</v>
       </c>
       <c r="G64" t="n">
-        <v>0.0005712509155273438</v>
+        <v>18.41884279251099</v>
       </c>
       <c r="H64" t="n">
         <v>0</v>
@@ -2110,16 +2110,16 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>0.0005609989166259766</v>
+        <v>16.04438877105713</v>
       </c>
       <c r="B65" t="n">
-        <v>1137.7734375</v>
+        <v>1127.921875</v>
       </c>
       <c r="C65" t="n">
-        <v>0</v>
+        <v>13.6</v>
       </c>
       <c r="D65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E65" t="n">
         <v>0</v>
@@ -2128,7 +2128,7 @@
         <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>0.0005600452423095703</v>
+        <v>16.04438710212708</v>
       </c>
       <c r="H65" t="n">
         <v>0</v>
@@ -2136,16 +2136,16 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>0.0005850791931152344</v>
+        <v>14.9456148147583</v>
       </c>
       <c r="B66" t="n">
-        <v>1137.7734375</v>
+        <v>1127.92578125</v>
       </c>
       <c r="C66" t="n">
-        <v>0</v>
+        <v>13.6</v>
       </c>
       <c r="D66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E66" t="n">
         <v>0</v>
@@ -2154,7 +2154,7 @@
         <v>0</v>
       </c>
       <c r="G66" t="n">
-        <v>0.000583648681640625</v>
+        <v>14.94561266899109</v>
       </c>
       <c r="H66" t="n">
         <v>0</v>
@@ -2162,16 +2162,16 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>0.0005509853363037109</v>
+        <v>14.73616552352905</v>
       </c>
       <c r="B67" t="n">
-        <v>1137.7734375</v>
+        <v>1127.92578125</v>
       </c>
       <c r="C67" t="n">
-        <v>0</v>
+        <v>14.5</v>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E67" t="n">
         <v>0</v>
@@ -2180,7 +2180,7 @@
         <v>0</v>
       </c>
       <c r="G67" t="n">
-        <v>0.0005495548248291016</v>
+        <v>14.73616337776184</v>
       </c>
       <c r="H67" t="n">
         <v>0</v>
@@ -2188,16 +2188,16 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>0.0006215572357177734</v>
+        <v>44.47607326507568</v>
       </c>
       <c r="B68" t="n">
-        <v>1137.77734375</v>
+        <v>1127.9296875</v>
       </c>
       <c r="C68" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E68" t="n">
         <v>0</v>
@@ -2206,7 +2206,7 @@
         <v>0</v>
       </c>
       <c r="G68" t="n">
-        <v>0.0006206035614013672</v>
+        <v>44.47607064247131</v>
       </c>
       <c r="H68" t="n">
         <v>0</v>

</xml_diff>